<commit_message>
Refactor test automation script and update README for new URL and file structure
</commit_message>
<xml_diff>
--- a/IT23713680.xlsx
+++ b/IT23713680.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -439,7 +439,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="18.7109375" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
+    <col width="29.5703125" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -506,7 +512,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ඔයා මොකද කරන්නේ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -548,7 +554,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>කොහොමද සපා ස්නිප</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -590,7 +596,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ඉක්මන එන්න කියන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -632,7 +638,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>මෙතන නවත්තන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -674,7 +680,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>මට කතා කරන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -716,7 +722,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>මට කතා කරන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -758,7 +764,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>සුබම සුබ දවසක්</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -800,7 +806,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>කොහොම හරි කරන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -842,7 +848,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>කොහොම හරි කරන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -884,7 +890,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>හෙට set වෙමුද???</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -926,7 +932,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>අපි අපේ රටට ආදරේ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -968,7 +974,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ඔයා ඔතෙන්ට් යන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1010,7 +1016,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ඔයා ඔතෙන්ට් යන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1052,7 +1058,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>අද full happy</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1094,7 +1100,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>අද full happy</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1136,7 +1142,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>take care මචන්</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1178,7 +1184,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>මගේ password මොකක්ද</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1220,7 +1226,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>wifi signal නෑනේ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1262,7 +1268,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>wifi signal නෑනේ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1304,7 +1310,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>zoom link එක එවන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1346,7 +1352,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>මට NIC ඒක දාන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1388,7 +1394,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>මට NIC ඒක දාන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1430,7 +1436,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ASAP assignment එක දාන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1472,7 +1478,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ලබ් එකේ වැඩ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1514,7 +1520,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ලබ් එකේ වැඩ</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1556,7 +1562,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>අපි kandy යමුද</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1598,7 +1604,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ගාල්ලේ ෆේස් set වෙමු</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1640,7 +1646,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>අමිල මාව දැක්කද</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1682,7 +1688,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>මට 500ක් දාන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1724,7 +1730,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2nd floor එක</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1766,7 +1772,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2nd floor එක</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1808,7 +1814,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Rs. 1000ක් දාන්න</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1850,7 +1856,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>EUR 50 කීයක්ද</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1890,7 +1896,11 @@
           <t>12.00noon පිටත් වේවි.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -1930,7 +1940,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>12.00noon පිටත් වේවි</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1970,7 +1980,11 @@
           <t>2026-05-05 අවසාන දිනය.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2010,7 +2024,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-05-05 deadline</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2050,7 +2064,11 @@
           <t>කිලෝ 10ක් බරයි.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2090,7 +2108,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>10kg බරයි</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2130,7 +2148,11 @@
           <t>මාර කට්ටක් කෑවේ.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2168,7 +2190,11 @@
           <t>ලින්ක් එක: www.test.com</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2206,7 +2232,11 @@
           <t>ඊමේල් එක: abc@gmail.com</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2244,7 +2274,11 @@
           <t>මාව මතකද? 🙂</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2282,7 +2316,11 @@
           <t>එපා වෙනවා 😡</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2320,7 +2358,11 @@
           <t>හරි හරි, යමු.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2358,7 +2400,11 @@
           <t>නියමයි බ්‍රෝ!</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2398,7 +2444,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>නියමයි bro!</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2438,7 +2484,11 @@
           <t>1st place ගත්තා.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -2478,7 +2528,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Colombo bus එක</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2520,7 +2570,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Colombo bus එක</t>
+          <t>ERROR</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">

</xml_diff>

<commit_message>
Refactor test automation script to simplify code and improve readability
</commit_message>
<xml_diff>
--- a/IT23713680.xlsx
+++ b/IT23713680.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -439,13 +439,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="18.7109375" customWidth="1" min="3" max="3"/>
-    <col width="57" customWidth="1" min="4" max="4"/>
-    <col width="29.5703125" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -497,22 +491,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>oya mwd krnne</t>
+          <t>oya kohomada exam ekata ready wenne?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ඔයා මොනවද කරන්නේ?</t>
+          <t>ඔයා කොහොමද exam එකට ready වෙන්නේ?</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඔය කොහොමඩ එxඅම් එකට රේඩ්ය් wඑන්නෙ?</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -527,7 +521,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Rationale: System fails to recognize 'mwd' as 'monawada'</t>
+          <t>Evidence: The overall message is a question containing "?"</t>
         </is>
       </c>
     </row>
@@ -539,22 +533,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>khmda sapa snipa</t>
+          <t>ai oya me dawaswala wada wadi kiyanne?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>කොහොමද සැප සනීප?</t>
+          <t>ඇයි ඔයා මේ දවස්වල වැඩ වැඩී කියන්නේ?</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඓ ඔය මෙ ඩwඅසwඅල wඅඩ wඅඩි කියන්නෙ?</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -569,7 +563,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rationale: System fails to recognize 'khmda'</t>
+          <t>Evidence: "ai oya" indicates a question structure.</t>
         </is>
       </c>
     </row>
@@ -586,17 +580,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ikmna enna kiynna</t>
+          <t>mata wahama e file eka ewanna.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ඉක්මනින් එන්න කියන්න.</t>
+          <t>මට වහාම ඒ file එක එවන්න.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මට wඅහම එ ෆිලෙ එක එwඅන්න.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -611,7 +605,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Rationale: 'ikmna' and 'kiynna' are clipped forms</t>
+          <t>Evidence: "wahama e file eka ewanna" is a direct command.</t>
         </is>
       </c>
     </row>
@@ -623,22 +617,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>methana nawaththann</t>
+          <t>karunakara wahanaya methanin aiyin karanna.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>මෙතන නවත්තන්න.</t>
+          <t>කරුණාකර වාහනය මෙතනින් අයින් කරන්න.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>කරුනකර wඅහනය මෙතනින් ඓයින් කරන්න.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -653,7 +647,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rationale: Clipped form 'nawaththann'</t>
+          <t>Evidence: Uses "karunakara" to give an instruction.</t>
         </is>
       </c>
     </row>
@@ -670,17 +664,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>mta katha krnn</t>
+          <t>subha udasanak wewa hamotama!</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>මට කතා කරන්න.</t>
+          <t>සුභ උදෑසනක් වේවා හැමෝටම!</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>සුබ්හ උඩසනක් wඑwඅ හමොටම!</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -690,12 +684,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Rationale: Common chat shorthand 'mta', 'krnn'</t>
+          <t>Evidence: "subha udasanak" is a morning greeting.</t>
         </is>
       </c>
     </row>
@@ -712,17 +706,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>poddak help krnn</t>
+          <t>niwadu dawasema sapa weewa!</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>පොඩ්ඩක් උදව් කරන්න.</t>
+          <t>නිවාඩු දවසේම සැප වේවා!</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>නිwඅඩු ඩwඅසෙම සප wඒwඅ!</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -732,12 +726,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Rationale: Mixed English word 'help' with clipped Sinhala</t>
+          <t>Evidence: Greeting for a holiday.</t>
         </is>
       </c>
     </row>
@@ -749,22 +743,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>subama suba dawsak</t>
+          <t>oyata puluwannam mage assignment eka balanna.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>සුබම සුබ දවසක්!</t>
+          <t>ඔයාට පුළුවන්නම් මගේ assignment එක බලන්න.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඔයට පුලුwඅන්නම් මගෙ අස්සිග්න්මෙන්ට් එක බලන්න.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -774,12 +768,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Rationale: Variation in 'dawsak'</t>
+          <t>Evidence: "puluwannam... balanna" makes a request.</t>
         </is>
       </c>
     </row>
@@ -791,22 +785,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kohoma hari krnn</t>
+          <t>ane poddak e form eka fill karala dennako.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>කොහොම හරි කරන්න.</t>
+          <t>අනේ පොඩ්ඩක් ඒ form එක fill කරලා දෙන්නකෝ.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අනෙ පොඩ්ඩක් එ ෆොර්ම් එක ෆිල්ල් කරල ඩෙන්නකො.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -816,12 +810,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Repeated words</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rationale: 'krnn' fails in repeated context</t>
+          <t>Evidence: "ane poddak... dennako" is a pleading request.</t>
         </is>
       </c>
     </row>
@@ -838,17 +832,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>heta set wemuda???</t>
+          <t>ow, mama eka heta karannam.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>හෙට සෙට් වෙමුද?</t>
+          <t>ඔව්, මම ඒක හෙට කරන්නම්.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඔw, මම එක හෙට කරන්නම්.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -858,12 +852,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Rationale: Excessive question marks often break transliterators</t>
+          <t>Evidence: Starts with "ow" (yes) indicating a response.</t>
         </is>
       </c>
     </row>
@@ -880,17 +874,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>mchn! mwa mtkd?</t>
+          <t>na, mata eka karanna wenne na.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>මචං! මාව මතකද?</t>
+          <t>නෑ, මට ඒක කරන්න වෙන්නේ නෑ.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>න, මට එක කරන්න wඑන්නෙ න.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -900,12 +894,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Rationale: Exclamation marks and chat slang combined</t>
+          <t>Evidence: Starts with "na" (no) as a response.</t>
         </is>
       </c>
     </row>
@@ -917,22 +911,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>api ape ratata adree</t>
+          <t>eka nam ithin digatama digatama wena deyak.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>අපි අපේ රටට ආදරෙයි.</t>
+          <t>ඒක නම් ඉතින් දිගටම දිගටම වෙන දෙයක්.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>එක නම් ඉතින් ඩිගටම ඩිගටම wඑන ඩෙයක්.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -942,12 +936,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Romanization / Spelling Variants</t>
+          <t>Repeated Words</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Rationale: 'adree' is a non-standard phonetic spelling</t>
+          <t>Evidence: "digatama digatama" is repeated.</t>
         </is>
       </c>
     </row>
@@ -964,17 +958,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>oya othent ynn</t>
+          <t>hemin hemin gihin wede karamu.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ඔයා ඔතනට යන්න.</t>
+          <t>හෙමින් හෙමින් ගිහින් වැඩේ කරමු.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>හෙමින් හෙමින් ගිහින් wඑඩෙ කරමු.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -984,12 +978,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Romanization / Spelling Variants</t>
+          <t>Repeated Words</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Rationale: 'othent' for 'othanata'</t>
+          <t>Evidence: "hemin hemin" indicates slow repetition.</t>
         </is>
       </c>
     </row>
@@ -1001,22 +995,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>mchn oya busy da?</t>
+          <t>mama yanna haduwe... eth oya awane!</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>මචං ඔයා බිසී ද?</t>
+          <t>මම යන්න හැදුවේ... ඒත් ඔයා ආවනේ!</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මම යන්න හඩුwඑ... එත් ඔය අwඅනෙ!</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1026,12 +1020,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions in Singlish</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Rationale: 'busy' may not transliterate to 'බිසී'</t>
+          <t>Evidence: Uses ellipsis "..." and exclamation "!".</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1042,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>adha full happy</t>
+          <t>mokak? eka wenna baha!</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>අද ෆුල් හැපි.</t>
+          <t>මොකක්? ඒක වෙන්න බැහැ!</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මොකක්? එක wඑන්න බහ!</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1068,12 +1062,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions in Singlish</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Rationale: 'full' and 'happy' are common chat insertions</t>
+          <t>Evidence: Uses "?" and "!".</t>
         </is>
       </c>
     </row>
@@ -1085,22 +1079,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>api den on the way enwa</t>
+          <t>mama gedra yanwa passe dennm.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>අපි දැන් on the way එනවා.</t>
+          <t>මම ගෙදර යනවා පස්සේ දෙන්නම්.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මම ගෙඩ්‍ර යනwඅ පස්සෙ ඩෙන්න්ම්.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1110,12 +1104,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases in Singlish</t>
+          <t>Romanization / Spelling Variants</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Rationale: Phrases like 'on the way' should remain English</t>
+          <t>Evidence: "gedra" instead of gedara, "yanwa" instead of yanawa.</t>
         </is>
       </c>
     </row>
@@ -1127,22 +1121,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>take care mchn</t>
+          <t>eka nkn boruwak wge neda?</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ටේක් කෙයාර් මචං.</t>
+          <t>ඒක නිකන් බොරුවක් වගේ නේද?</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>එක න්ක්න් බොරුwඅක් wගෙ නෙඩ?</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1152,12 +1146,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases in Singlish</t>
+          <t>Romanization / Spelling Variants</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Rationale: Conversational English phrases</t>
+          <t>Evidence: "nkn" instead of nikan, "wge" instead of wage.</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1163,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>mage password mkkd</t>
+          <t>ape aluth car eka harima lassanai.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>මගේ password මොකක්ද?</t>
+          <t>අපේ අලුත් car එක හරිම ලස්සනයි.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අපෙ අලුත් cඅර් එක හරිම ලස්සනෛ.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1194,12 +1188,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>English Digital Terms in Singlish</t>
+          <t>Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Rationale: Digital term 'password'</t>
+          <t>Evidence: The English word "car" is inserted.</t>
         </is>
       </c>
     </row>
@@ -1216,17 +1210,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>wifi signal nane</t>
+          <t>oyage phone eka weda nadda?</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>වයිෆයි සිග්නල් නෑනේ.</t>
+          <t>ඔයාගේ phone එක වැඩ නැද්ද?</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඔයගෙ ප්හොනෙ එක wඑඩ නඩ්ඩ?</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1236,12 +1230,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>English Digital Terms in Singlish</t>
+          <t>Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Rationale: Technical term 'wifi'</t>
+          <t>Evidence: "phone" is inserted.</t>
         </is>
       </c>
     </row>
@@ -1253,22 +1247,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>zoom link eka ewnn</t>
+          <t>mama ada all day working eken inne.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Zoom link එක එවන්න.</t>
+          <t>මම අද all day working එකෙන් ඉන්නේ.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මම අඩ අල්ල් ඩය් wඔර්කින්ග් එකෙන් ඉන්නේ.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1278,12 +1272,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Platform/App Names in Singlish</t>
+          <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Rationale: App name 'zoom'</t>
+          <t>Evidence: "all day working" is a multi-word phrase.</t>
         </is>
       </c>
     </row>
@@ -1295,22 +1289,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>fb eke dkpuda</t>
+          <t>api next week on vacation yanawa.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>FB එකේ දැක්කාද?</t>
+          <t>අපි next week on vacation යනවා.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අපි නෙxට් wඒක් ඔන් වcඅටිඔන් යනwඅ.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1320,12 +1314,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Platform/App Names in Singlish</t>
+          <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Rationale: Platform abbreviation 'fb'</t>
+          <t>Evidence: "next week on vacation" is a phrase.</t>
         </is>
       </c>
     </row>
@@ -1337,22 +1331,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>mta NIC eka dnn</t>
+          <t>oya software update eka daagaththada?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>මට NIC එක දෙන්න.</t>
+          <t>ඔයා software update එක දාගත්තද?</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඔය සොෆ්ටwඅරෙ උප්ඩටෙ එක ඩාගත්තඩ?</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1362,12 +1356,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
+          <t>English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Rationale: Acronym 'NIC'</t>
+          <t>Evidence: "software update" is a digital term.</t>
         </is>
       </c>
     </row>
@@ -1379,22 +1373,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ASAP assignment eka dnn</t>
+          <t>mage router eke aulak thiyenawa.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ASAP assignment එක දෙන්න.</t>
+          <t>මගේ router එකේ අවුලක් තියෙනවා.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මගෙ රොඋටෙර් එකෙ ඖලක් තියෙනwඅ.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1404,12 +1398,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
+          <t>English Digital Terms in Singlish</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Rationale: Professional abbreviation 'ASAP'</t>
+          <t>Evidence: "router" is a digital/networking term.</t>
         </is>
       </c>
     </row>
@@ -1421,22 +1415,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>heta exam mchn</t>
+          <t>mata Instagram eken request ekak awa.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>හෙට exam මචං.</t>
+          <t>මට Instagram එකෙන් request එකක් ආවා.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මට ඉන්ස්ටග්‍රම් එකෙන් රෙqඋඑස්ට් එකක් අwඅ.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1446,12 +1440,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>English Clipped Forms in Singlish</t>
+          <t>Platform/App Names in Singlish</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Rationale: Clipped English word 'exam'</t>
+          <t>Evidence: "Instagram" is an app name.</t>
         </is>
       </c>
     </row>
@@ -1463,22 +1457,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>lab eke weda</t>
+          <t>TikTok eke e video eka viral gihin.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>lab එකේ වැඩ.</t>
+          <t>TikTok එකේ ඒ video එක viral ගිහින්.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඨික්ඨොක් එකෙ එ විඩෙඔ එක විරල් ගිහින්.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1488,12 +1482,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>English Clipped Forms in Singlish</t>
+          <t>Platform/App Names in Singlish</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Rationale: Clipped word 'lab'</t>
+          <t>Evidence: "TikTok" is a platform name.</t>
         </is>
       </c>
     </row>
@@ -1510,17 +1504,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>api kandy yamuda</t>
+          <t>mage CV eka oyata ewwa.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>අපි මහනුවර යමුද?</t>
+          <t>මගේ CV එක ඔයාට එව්වා.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මගෙ CV එක ඔයට එwwඅ.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1530,12 +1524,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Place Names Embedded in Singlish</t>
+          <t>English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Rationale: Common place name 'kandy'</t>
+          <t>Evidence: "CV" is an acronym.</t>
         </is>
       </c>
     </row>
@@ -1552,17 +1546,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>galle face set wemu</t>
+          <t>API eka down wela wage.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Galle Face සෙට් වෙමු.</t>
+          <t>API එක down වෙලා වගේ.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>API එක ඩොwන් wඑල wඅගෙ.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1572,12 +1566,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Place Names Embedded in Singlish</t>
+          <t>English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Rationale: Multi-word place name</t>
+          <t>Evidence: "API" is an abbreviation/acronym.</t>
         </is>
       </c>
     </row>
@@ -1594,17 +1588,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>amila mwa dkd</t>
+          <t>api uni gihin katha karamu.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>අමිල මාව දැක්කාද?</t>
+          <t>අපි uni ගිහින් කතා කරමු.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අපි උනි ගිහින් කත කරමු.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1614,12 +1608,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Person Names Embedded in Singlish</t>
+          <t>English Clipped Forms in Singlish</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Rationale: Common name 'Amila'</t>
+          <t>Evidence: "uni" is a clipped form of university.</t>
         </is>
       </c>
     </row>
@@ -1636,17 +1630,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>nirmal ada awe na</t>
+          <t>mama lab ekata yanna hadanne.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>නිර්මල් අද ආවේ නෑ.</t>
+          <t>මම lab එකට යන්න හදන්නේ.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මම ලබ් එකට යන්න හඩන්නෙ.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1656,12 +1650,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Person Names Embedded in Singlish</t>
+          <t>English Clipped Forms in Singlish</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Rationale: Common name 'Nirmal'</t>
+          <t>Evidence: "lab" is a clipped form of laboratory.</t>
         </is>
       </c>
     </row>
@@ -1678,17 +1672,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>mta 500k dnn</t>
+          <t>api Kandy trip ekak yanawada?</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>මට 500ක් දෙන්න.</t>
+          <t>අපි Kandy trip එකක් යනවාද?</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අපි ඛන්ඩ්ය් ට්‍රිප් එකක් යනwඅඩ?</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1698,12 +1692,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>Place Names Embedded in Singlish</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Rationale: Suffix 'k' after number</t>
+          <t>Evidence: "Kandy" is a place name.</t>
         </is>
       </c>
     </row>
@@ -1720,17 +1714,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2nd floor eka</t>
+          <t>ada Colombo traffic wadi wage.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2nd floor එක.</t>
+          <t>අද Colombo traffic වැඩි වගේ.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අඩ Cඔලොම්බො ට්‍රෆ්ෆිc wඅඩි wඅගෙ.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1740,12 +1734,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>Place Names Embedded in Singlish</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Rationale: Ordinal number suffix 'nd'</t>
+          <t>Evidence: "Colombo" is a place name.</t>
         </is>
       </c>
     </row>
@@ -1757,22 +1751,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Rs. 1000k dnn</t>
+          <t>Kamal ayya heta gedara enawalu.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>රුපියල් 1000ක් දෙන්න.</t>
+          <t>කමල් අයියා හෙට ගෙදර එනවාලු.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ඛමල් අය්ය හෙට ගෙඩර එනwඅලු.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1782,12 +1776,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>Person Names Embedded in Singlish</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Rationale: Currency symbol 'Rs.'</t>
+          <t>Evidence: "Kamal" is a person's name.</t>
         </is>
       </c>
     </row>
@@ -1799,22 +1793,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EUR 50 kiykda</t>
+          <t>Nimal ekka katha karala balanna.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EUR 50 කීයක්ද?</t>
+          <t>නිමල් එක්ක කතා කරලා බලන්න.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ණිමල් එක්ක කත කරල බලන්න.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1824,12 +1818,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>Person Names Embedded in Singlish</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Rationale: Foreign currency 'EUR'</t>
+          <t>Evidence: "Nimal" is a person's name.</t>
         </is>
       </c>
     </row>
@@ -1846,17 +1840,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>welawa 8.30am</t>
+          <t>lamayi 10denekma mekata awith.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>වෙලාව 8.30am.</t>
+          <t>ළමයි 10දෙනෙක්ම මේකට ඇවිත්.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ලමයි 10ඩෙනෙක්ම මෙකට අwඉත්.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1866,12 +1860,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Rationale: Time suffix 'am'</t>
+          <t>Evidence: "10denekma" contains a number with a numeric suffix.</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1882,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>12.00noon pitath wewi</t>
+          <t>eka 2weni wathawatath wuna.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>12.00noon පිටත් වේවි.</t>
+          <t>ඒක 2වෙනි වතාවටත් වුණා.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>එක 2wඑනි wඅතwඅටත් wඋන.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1908,12 +1902,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Rationale: Word-based time format 'noon'</t>
+          <t>Evidence: "2weni" contains a number and suffix.</t>
         </is>
       </c>
     </row>
@@ -1930,17 +1924,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>heta Feb 14 ne</t>
+          <t>meka Rs. 1500k withara wenawa.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>හෙට පෙබරවාරි 14 නේ.</t>
+          <t>මේක Rs. 1500ක් විතර වෙනවා.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මෙක Rස්. 1500ක් wඉතර wඑනwඅ.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1950,12 +1944,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Rationale: Abbreviated month 'Feb'</t>
+          <t>Evidence: Contains "Rs. 1500k".</t>
         </is>
       </c>
     </row>
@@ -1972,17 +1966,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-05-05 deadline</t>
+          <t>mata USD 50k transfer karanna.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-05-05 අවසාන දිනය.</t>
+          <t>මට USD 50ක් transfer කරන්න.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මට USD 50ක් ට්‍රන්ස්ෆෙර් කරන්න.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1992,12 +1986,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Rationale: ISO date format</t>
+          <t>Evidence: Contains "USD 50k".</t>
         </is>
       </c>
     </row>
@@ -2009,22 +2003,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>adi 5k usa</t>
+          <t>meeting eka 10:00AM walata thiyenne.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>අඩි 5ක් උස.</t>
+          <t>meeting එක 10:00AM වලට තියෙන්නේ.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මේටින්ග් එක 10:00AM wඅලට තියෙන්නෙ.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2034,12 +2028,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Rationale: Measurement 'adi' (feet)</t>
+          <t>Evidence: Contains time format "10:00AM".</t>
         </is>
       </c>
     </row>
@@ -2056,17 +2050,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10kg barayi</t>
+          <t>api 5.30pm weddi meken yamu.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>කිලෝ 10ක් බරයි.</t>
+          <t>අපි 5.30pm වෙද්දී මේකෙන් යමු.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>අපි 5.30pm wඑඩ්ඩි මෙකෙන් යමු.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2076,12 +2070,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Rationale: Abbreviated unit 'kg'</t>
+          <t>Evidence: Contains time format "5.30pm".</t>
         </is>
       </c>
     </row>
@@ -2093,22 +2087,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sirawata elakiri mchn</t>
+          <t>mage birthday eka 2026-05-12 thiyenne.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>සිරාවට එළකිරි මචං.</t>
+          <t>මගේ birthday එක 2026-05-12 තියෙන්නේ.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මගෙ බිර්ත්ඩය් එක 2026-05-12 තියෙන්නෙ.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2118,12 +2112,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Rationale: Heavy use of slang</t>
+          <t>Evidence: Contains date "2026-05-12".</t>
         </is>
       </c>
     </row>
@@ -2135,22 +2129,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>mara kattak kawe</t>
+          <t>project submission eka March 15 daana.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>මාර කට්ටක් කෑවේ.</t>
+          <t>project submission එක March 15 දාන.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>ප්‍රොජෙcට් සුබ්මිස්සිඔන් එක මර්ච් 15 ඩාන.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2160,12 +2154,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Rationale: Figurative slang</t>
+          <t>Evidence: Contains date format "March 15".</t>
         </is>
       </c>
     </row>
@@ -2177,22 +2171,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>link eka: www.test.com</t>
+          <t>mama 5kg withara bara ussuwa.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ලින්ක් එක: www.test.com</t>
+          <t>මම 5kg විතර බර ඉස්සුවා.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මම 5ක්ග් wඉතර බර උස්සුwඅ.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2202,12 +2196,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Online Identifiers in Singlish</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Rationale: URL recognition</t>
+          <t>Evidence: Contains unit "5kg".</t>
         </is>
       </c>
     </row>
@@ -2219,22 +2213,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>email eka: abc@gmail.com</t>
+          <t>meka aduma 10m digai.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ඊමේල් එක: abc@gmail.com</t>
+          <t>මේක අඩුම 10m දිගයි.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මෙක අඩුම 10ම් ඩිගෛ.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2244,12 +2238,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Online Identifiers in Singlish</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Rationale: Email address format</t>
+          <t>Evidence: Contains measurement unit "10m".</t>
         </is>
       </c>
     </row>
@@ -2261,22 +2255,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>mwa mtkd? 🙂</t>
+          <t>patta machan, elakiri wage weda.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>මාව මතකද? 🙂</t>
+          <t>පට්ට මචන්, එළකිරි වගේ වැඩ.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>පට්ට මචන්, එලකිරි wඅගෙ wඑඩ.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2286,12 +2280,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Inputs Containing Emojis</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Rationale: Emoji handling</t>
+          <t>Evidence: "patta" and "elakiri" are slangs.</t>
         </is>
       </c>
     </row>
@@ -2308,17 +2302,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>epa wenwa 😡</t>
+          <t>uba mara porakne ban.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>එපා වෙනවා 😡</t>
+          <t>උඹ මාර පොරක්නේ බන්.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>උබ මර පොරක්නෙ බන්.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2328,12 +2322,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Inputs Containing Emojis</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Rationale: Angry emoji</t>
+          <t>Evidence: "uba mara porakne ban" is heavy casual slang.</t>
         </is>
       </c>
     </row>
@@ -2345,22 +2339,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>hari hari, ymu</t>
+          <t>mata me file eka admin@sliit.lk ekata email karanna.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>හරි හරි, යමු.</t>
+          <t>මට මේ file එක admin@sliit.lk එකට email කරන්න.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මට මෙ ෆිලෙ එක අඩ්මින්@ස්ලීට්.ල්ක් එකට එමෛල් කරන්න.</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2370,12 +2364,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Repeated words</t>
+          <t>Online Identifiers in Singlish</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Rationale: Punctuation between repeated words</t>
+          <t>Evidence: Contains email address "admin@sliit.lk".</t>
         </is>
       </c>
     </row>
@@ -2387,22 +2381,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>niyamayi bro!</t>
+          <t>website eka www.mytest.com balanna.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>නියමයි බ්‍රෝ!</t>
+          <t>website එක www.mytest.com බලන්න.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>wඑබ්සිටෙ එක www.ම්ය්ටෙස්ට්.cඔම් බලන්න.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2412,12 +2406,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Online Identifiers in Singlish</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Rationale: Casual English insertion 'bro'</t>
+          <t>Evidence: Contains URL "www.mytest.com".</t>
         </is>
       </c>
     </row>
@@ -2434,17 +2428,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>@Kamal mtkd meka?</t>
+          <t>mata nam hari sathutui ada 😊</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>@Kamal මතකද මේක?</t>
+          <t>මට නම් හරි සතුටුයි අද 😊</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මට නම් හරි සතුටුඉ අඩ 😊</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2454,12 +2448,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Online Identifiers in Singlish</t>
+          <t>Inputs Containing Emojis</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Rationale: Social media handle symbol '@'</t>
+          <t>Evidence: Contains the 😊 emoji.</t>
         </is>
       </c>
     </row>
@@ -2476,17 +2470,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1st place gaththa</t>
+          <t>eka nam patta joke eka 😂</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1st place ගත්තා.</t>
+          <t>ඒක නම් පට්ට joke එක 😂</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>එක නම් පට්ට ජොකෙ එක 😂</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2496,12 +2490,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>Inputs Containing Emojis</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Rationale: Ranking suffix 'st'</t>
+          <t>Evidence: Contains the 😂 emoji.</t>
         </is>
       </c>
     </row>
@@ -2513,22 +2507,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Colombo bus eka</t>
+          <t>machan, heta ude 8:30AM weddhi meeting ekata enna puluwanda? ape project eka gena katha karanna one. sir kiwwa ASAP report eka submit karanna kiyala. oyage part eka iwara nam mata email ekak danna student2026@sliit.lk ekata. nathnam WhatsApp eken message ekak danna puluwanne. mama Kandy idala enne, so Colombo traffic eke hira weyi kiyala bayai. anyway api try karamu wede iwara karanna. godak un kattak kala weda kale, so we need to get 100 marks out of this. ok boss, see you tomorrow! 😂👍</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>කොළඹ බස් එක.</t>
+          <t>මචන්, හෙට උදේ 8:30AM වෙද්දී meeting එකට එන්න පුළුවන්ද? අපේ project එක ගැන කතා කරන්න ඕනේ. sir කිව්වා ASAP report එක submit කරන්න කියලා. ඔයාගේ part එක ඉවර නම් මට email එකක් දාන්න student2026@sliit.lk එකට. නැත්නම් WhatsApp එකෙන් message එකක් දාන්න පුළුවන්නේ. මම Kandy ඉදලා එන්නේ, so Colombo traffic එකේ හිර වෙයි කියලා බයයි. anyway අපි try කරමු වැඩේ ඉවර කරන්න. ගොඩක් උන් කට්ටක් කාලා වැඩ කළේ, so we need to get 100 marks out of this. ok boss, see you tomorrow! 😂👍</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>මචන්, හෙට උඩෙ 8:30AM wඑඩ්දි මේටින්ග් එකට එන්න පුලුwඅන්ඩ? අපෙ ප්‍රොජෙcට් එක ගෙන කත කරන්න ඔනෙ. සිර් කිwwඅ ASAP රෙපොර්ට් එක සුබ්මිට් කරන්න කියල. ඔයගෙ පර්ට් එක ඉwඅර නම් මට එමෛල් එකක් ඩන්න ස්ටුඩෙන්ට්2026@ස්ලීට්.ල්ක් එකට. නත්නම් Wහට්සප්ප් එකෙන් මෙස්සගෙ එකක් ඩන්න පුලුwඅන්නෙ. මම ඛන්ඩ්ය් ඉඩල එන්නෙ, සො Cඔලොම්බො ට්‍රෆ්ෆිc එකෙ හිර wඑයි කියල බයෛ. අන්යwඅය් අපි ට්‍රය් කරමු wඑඩෙ ඉwඅර කරන්න. ගොඩක් උන් කට්ටක් කල wඑඩ කලෙ, සො wඑ නේඩ් ටො ගෙට් 100 මර්ක්ස් ඔ</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2538,12 +2532,15 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Place Names Embedded in Singlish</t>
+          <t>Inputs Containing Emojis
+Online Identifiers in Singlish
+Inputs with Time Formats
+English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Rationale: Capital city name</t>
+          <t>Rationale: L-size string. Contains time '8:30AM', acronym 'ASAP', email 'student2026@sliit.lk', apps 'WhatsApp', places 'Kandy', 'Colombo', and emojis '😂👍'.</t>
         </is>
       </c>
     </row>
@@ -2555,22 +2552,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ayubovan sematama</t>
+          <t>hello yaluwane! oyalage assignment eka complete kalada? mage eka nam thaama 50% witharai iwara wela thiyenne. me dawaswala godak busy nisa eka digatama karanna wela na. Rs. 2500k deela internet package ekakuth gaththa zoom sessions wala inna one nisa. kohoma hari 2026-05-05 weddi okkoma iwara karala submit karanna thiyenawa. oyala danna kenek innawanam mata me part ekata udaw karanna kiyala poddak kiyannako. mycontact@email.com ekata mail ekak damma kiyala kiyanna. thuthi! 🙏✨</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ආයුබෝවන් සැමටම.</t>
+          <t>hello යාලුවනේ! ඔයාලගේ assignment එක complete කළාද? මගේ එක නම් තාම 50% විතරයි ඉවර වෙලා තියෙන්නේ. මේ දවස්වල ගොඩක් busy නිසා එක දිගටම කරන්න වෙලා නෑ. Rs. 2500ක් දීලා internet package එකකුත් ගත්තා zoom sessions වල ඉන්න ඕනේ නිසා. කොහොම හරි 2026-05-05 වෙද්දී ඔක්කොම ඉවර කරලා submit කරන්න තියෙනවා. ඔයාලා දන්න කෙනෙක් ඉන්නවනම් මට මේ part එකට උදව් කරන්න කියලා පොඩ්ඩක් කියන්නකෝ. mycontact@email.com එකට mail එකක් දැම්මා කියලා කියන්න. ස්තුතියි! 🙏✨</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>හෙල්ලො යලුwඅනෙ! ඔයලගෙ අස්සිග්න්මෙන්ට් එක cඔම්ප්ලෙටෙ කලඩ? මගෙ එක නම් තාම 50% wඉතරෛ ඉwඅර wඑල තියෙන්නෙ. මෙ ඩwඅසwඅල ගොඩක් බුස්ය් නිස එක ඩිගටම කරන්න wඑල න. Rස්. 2500ක් ඩේල ඉන්ටෙර්නෙට් පcකගෙ එකකුත් ගත්ත zඕම් සෙස්සිඔන්ස් wඅල ඉන්න ඔනෙ නිස. කොහොම හරි 2026-05-05 wඑඩ්ඩි ඔක්කොම ඉwඅර කරල සුබ්මිට් කරන්න තියෙනwඅ. ඔයල ඩන්න කෙනෙක් ඉන්නwඅනම් මට මෙ පර්ට් එකට උඩw කරන්න කියල පොඩ්ඩක් කියන්නකො. ම්යcඔන්ටcට්@එමෛල්.cඔම් එකට මෛල් එකක් ඩ</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2580,12 +2577,15 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Online Identifiers in Singlish
+Inputs with Currency
+Inputs with Dates
+Inputs Containing Emojis</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Rationale: Formal greeting variant</t>
+          <t>Rationale: L-size string. Contains currency 'Rs. 2500k', date '2026-05-05', email 'mycontact@email.com', app 'zoom', and emojis '🙏✨'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update IT23713680.xlsx with new data and finished
</commit_message>
<xml_diff>
--- a/IT23713680.xlsx
+++ b/IT23713680.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanithNirmal\Desktop\IT23713680\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEE07E3-7045-4EA2-A2ED-FF52388FD314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A30396EF-5DF1-44A9-8003-54DEB336582B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="287">
   <si>
     <t>TC ID</t>
   </si>
@@ -37,9 +37,6 @@
     <t>Actual output</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Singlish input types covered</t>
   </si>
   <si>
@@ -379,9 +376,6 @@
     <t>අපි next week on vacation යනවා.</t>
   </si>
   <si>
-    <t>අපි නෙxට් wඒක් ඔන් වcඅටිඔන් යනwඅ.</t>
-  </si>
-  <si>
     <t>Evidence: "next week on vacation" is a phrase.</t>
   </si>
   <si>
@@ -394,9 +388,6 @@
     <t>ඔයා software update එක දාගත්තද?</t>
   </si>
   <si>
-    <t>ඔය සොෆ්ටwඅරෙ උප්ඩටෙ එක ඩාගත්තඩ?</t>
-  </si>
-  <si>
     <t>English Digital Terms in Singlish</t>
   </si>
   <si>
@@ -412,9 +403,6 @@
     <t>මගේ router එකේ අවුලක් තියෙනවා.</t>
   </si>
   <si>
-    <t>මගෙ රොඋටෙර් එකෙ ඖලක් තියෙනwඅ.</t>
-  </si>
-  <si>
     <t>Evidence: "router" is a digital/networking term.</t>
   </si>
   <si>
@@ -851,6 +839,15 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>machan, heta ude 8:30AM weddhi meeting ekata enna. project eka gena katha karanna one. sir kiwwa ASAP report eka submit karanna kiyala. oyage part eka iwara nam mata email ekak danna student2026@sliit.lk ekata. nathnam WhatsApp message ekak danna. mama Kandy idala enne, Colombo traffic eke hira weyi kiyala bayai. ok boss, see you! 😂👍</t>
+  </si>
+  <si>
+    <t>මචන්, හෙට උදේ 8:30AM වෙද්දී meeting එකට එන්න. project එක ගැන කතා කරන්න ඕනේ. sir කිව්වා ASAP report එක submit කරන්න කියලා. ඔයාගේ part එක ඉවර නම් මට email එකක් දාන්න student2026@sliit.lk එකට. නැත්නම් WhatsApp message එකක් දාන්න. මම Kandy ඉදලා එන්නේ, Colombo traffic එකේ හිර වෙයි කියලා බයයි. ok boss, see you! 😂👍</t>
+  </si>
+  <si>
+    <t>මචන්, හෙට උඩෙ 8:30AM wඑඩ්දි මේටින්ග් එකට එන්න. ප්‍රොජෙcට් එක ගෙන කත කරන්න ඔනෙ. සිර් කිwwඅ ASAP රෙපොර්ට් එක සුබ්මිට් කරන්න කියල. ඔයගෙ පර්ට් එක ඉwඅර නම් මට එමෛල් එකක් ඩන්න ස්ටුඩෙන්ට්2026@ස්ලීට්.ල්ක් එකට. නත්නම් Wහට්සප්ප් මෙස්සගෙ එකක් ඩන්න. මම ඛන්ඩ්ය් ඉඩල එන්නෙ, Cඔලොම්බො ට්‍රෆ්ෆිc එකෙ හිර wඑයි කියල බයෛ. ඔක් බොස්ස්, සේ යොඋ! 😂👍</t>
   </si>
   <si>
     <t>Inputs Containing Emojis
@@ -865,6 +862,15 @@
     <t>Neg_0050</t>
   </si>
   <si>
+    <t>hello yaluwane! assignment eka complete kalada? mage eka thaama 50% iwarai. godak busy nisa karanna wela na. Rs. 2500k deela internet package gaththa zoom session inna one nisa. 2026-05-05 weddi submit karanna thiyenawa. danna kenek innawanam udaw karanna. mycontact@email.com ekata mail ekak danna kiyanna. thuthi! 🙏✨</t>
+  </si>
+  <si>
+    <t>hello යාලුවනේ! assignment එක complete කළාද? මගේ එක තාම 50% ඉවරයි. ගොඩක් busy නිසා කරන්න වෙලා නෑ. Rs. 2500ක් දීලා internet package ගත්තා zoom session ඉන්න ඕනේ නිසා. 2026-05-05 වෙද්දී submit කරන්න තියෙනවා. දන්න කෙනෙක් ඉන්නවනම් උදව් කරන්න. mycontact@email.com එකට mail එකක් දාන්න කියන්න. ස්තුතියි! 🙏✨</t>
+  </si>
+  <si>
+    <t>හෙල්ලො යලුwඅනෙ! අස්සිග්න්මෙන්ට් එක cඔම්ප්ලෙටෙ කලඩ? මගෙ එක තාම 50% ඉwඅරෛ. ගොඩක් බුස්ය් නිස කරන්න wඑල න. Rස්. 2500ක් ඩේල ඉන්ටෙර්නෙට් පcකගෙ ගත්ත zඕම් සෙස්සිඔන් ඉන්න ඔනෙ නිස. 2026-05-05 wඑඩ්ඩි සුබ්මිට් කරන්න තියෙනwඅ. ඩන්න කෙනෙක් ඉන්නwඅනම් උඩw කරන්න. ම්යcඔන්ටcට්@එමෛල්.cඔම් එකට මෛල් එකක් ඩන්න කියන්න. තුති! 🙏✨</t>
+  </si>
+  <si>
     <t>Online Identifiers in Singlish
 Inputs with Currency
 Inputs with Dates
@@ -874,22 +880,13 @@
     <t>Rationale: L-size string. Contains currency 'Rs. 2500k', date '2026-05-05', email 'mycontact@email.com', app 'zoom', and emojis '🙏✨'.</t>
   </si>
   <si>
-    <t>hello යාලුවනේ! assignment එක complete කළාද? මගේ එක තාම 50% ඉවරයි. ගොඩක් busy නිසා කරන්න වෙලා නෑ. Rs. 2500ක් දීලා internet package ගත්තා zoom session ඉන්න ඕනේ නිසා. 2026-05-05 වෙද්දී submit කරන්න තියෙනවා. දන්න කෙනෙක් ඉන්නවනම් උදව් කරන්න. mycontact@email.com එකට mail එකක් දාන්න කියන්න. ස්තුතියි! 🙏✨</t>
-  </si>
-  <si>
-    <t>hello yaluwane! assignment eka complete kalada? mage eka thaama 50% iwarai. godak busy nisa karanna wela na. Rs. 2500k deela internet package gaththa zoom session inna one nisa. 2026-05-05 weddi submit karanna thiyenawa. danna kenek innawanam udaw karanna. mycontact@email.com ekata mail ekak danna kiyanna. thuthi! 🙏✨</t>
-  </si>
-  <si>
-    <t>හෙල්ලො යලුwඅනෙ! අස්සිග්න්මෙන්ට් එක cඔම්ප්ලෙටෙ කලඩ? මගෙ එක තාම 50% ඉwඅරෛ. ගොඩක් බුස්ය් නිස කරන්න wඑල න. Rස්. 2500ක් ඩේල ඉන්ටෙර්නෙට් පcකගෙ ගත්ත zඕම් සෙස්සිඔන් ඉන්න ඔනෙ නිස. 2026-05-05 wඑඩ්ඩි සුබ්මිට් කරන්න තියෙනwඅ. ඩන්න කෙනෙක් ඉන්නwඅනම් උඩw කරන්න. ම්යcඔන්ටcට්@එමෛල්.cඔම් එකට මෛල් එකක් ඩන්න කියන්න. තුති! 🙏✨</t>
-  </si>
-  <si>
-    <t>machan, heta ude 8:30AM weddhi meeting ekata enna. project eka gena katha karanna one. sir kiwwa ASAP report eka submit karanna kiyala. oyage part eka iwara nam mata email ekak danna student2026@sliit.lk ekata. nathnam WhatsApp message ekak danna. mama Kandy idala enne, Colombo traffic eke hira weyi kiyala bayai. ok boss, see you! 😂👍</t>
-  </si>
-  <si>
-    <t>මචන්, හෙට උඩෙ 8:30AM wඑඩ්දි මේටින්ග් එකට එන්න. ප්‍රොජෙcට් එක ගෙන කත කරන්න ඔනෙ. සිර් කිwwඅ ASAP රෙපොර්ට් එක සුබ්මිට් කරන්න කියල. ඔයගෙ පර්ට් එක ඉwඅර නම් මට එමෛල් එකක් ඩන්න ස්ටුඩෙන්ට්2026@ස්ලීට්.ල්ක් එකට. නත්නම් Wහට්සප්ප් මෙස්සගෙ එකක් ඩන්න. මම ඛන්ඩ්ය් ඉඩල එන්නෙ, Cඔලොම්බො ට්‍රෆ්ෆිc එකෙ හිර wඑයි කියල බයෛ. ඔක් බොස්ස්, සේ යොඋ! 😂👍</t>
-  </si>
-  <si>
-    <t>මචන්, හෙට උදේ 8:30AM වෙද්දී meeting එකට එන්න. project එක ගැන කතා කරන්න ඕනේ. sir කිව්වා ASAP report එක submit කරන්න කියලා. ඔයාගේ part එක ඉවර නම් මට email එකක් දාන්න student2026@sliit.lk එකට. නැත්නම් WhatsApp message එකක් දාන්න. මම Kandy ඉදලා එන්නේ, Colombo traffic එකේ හිර වෙයි කියලා බයයි. ok boss, see you! 😂👍</t>
+    <t>අපි නෙxට් wඒක් ඔන් වcඅටිඔන් යනwඅ.</t>
+  </si>
+  <si>
+    <t>ඔය සොෆ්ටwඅරෙ උප්ඩටෙ එක ඩාගත්තඩ?</t>
+  </si>
+  <si>
+    <t>මගෙ රොඋටෙර් එකෙ ඖලක් තියෙනwඅ.</t>
   </si>
 </sst>
 </file>
@@ -1258,6 +1255,7 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="4" max="4" width="104" customWidth="1"/>
     <col min="5" max="5" width="92" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1277,1314 +1275,1312 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="1"/>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
       <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
         <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>35</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
         <v>36</v>
       </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>37</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>41</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" t="s">
         <v>42</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>37</v>
-      </c>
-      <c r="H7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>45</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>46</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>48</v>
-      </c>
-      <c r="H8" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
         <v>50</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>51</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>52</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" t="s">
         <v>53</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>56</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>57</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>59</v>
-      </c>
-      <c r="H10" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
         <v>61</v>
       </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>62</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>63</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" t="s">
         <v>64</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>59</v>
-      </c>
-      <c r="H11" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
         <v>66</v>
       </c>
-      <c r="B12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>67</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
         <v>69</v>
       </c>
-      <c r="F12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>70</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="B13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>74</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>69</v>
+      </c>
+      <c r="H13" t="s">
         <v>75</v>
-      </c>
-      <c r="F13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" t="s">
-        <v>70</v>
-      </c>
-      <c r="H13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
         <v>77</v>
       </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>78</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>79</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" t="s">
         <v>80</v>
       </c>
-      <c r="F14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>81</v>
-      </c>
-      <c r="H14" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
         <v>83</v>
       </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>84</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>85</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" t="s">
         <v>86</v>
-      </c>
-      <c r="F15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" t="s">
-        <v>81</v>
-      </c>
-      <c r="H15" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
       </c>
-      <c r="B16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>89</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>90</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
         <v>91</v>
       </c>
-      <c r="F16" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>92</v>
-      </c>
-      <c r="H16" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" t="s">
         <v>94</v>
       </c>
-      <c r="B17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>95</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>96</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>91</v>
+      </c>
+      <c r="H17" t="s">
         <v>97</v>
-      </c>
-      <c r="F17" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" t="s">
-        <v>92</v>
-      </c>
-      <c r="H17" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
         <v>99</v>
       </c>
-      <c r="B18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>100</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>101</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" t="s">
         <v>102</v>
       </c>
-      <c r="F18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>103</v>
-      </c>
-      <c r="H18" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
         <v>105</v>
       </c>
-      <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>106</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>107</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" t="s">
+        <v>102</v>
+      </c>
+      <c r="H19" t="s">
         <v>108</v>
-      </c>
-      <c r="F19" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" t="s">
-        <v>103</v>
-      </c>
-      <c r="H19" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
         <v>110</v>
       </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>111</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>112</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" t="s">
         <v>113</v>
       </c>
-      <c r="F20" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>114</v>
-      </c>
-      <c r="H20" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>115</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
         <v>116</v>
       </c>
-      <c r="B21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>117</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
+        <v>284</v>
+      </c>
+      <c r="F21" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" t="s">
+        <v>113</v>
+      </c>
+      <c r="H21" t="s">
         <v>118</v>
-      </c>
-      <c r="E21" t="s">
-        <v>119</v>
-      </c>
-      <c r="F21" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" t="s">
-        <v>114</v>
-      </c>
-      <c r="H21" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>120</v>
+      </c>
+      <c r="D22" t="s">
         <v>121</v>
       </c>
-      <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
+        <v>285</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" t="s">
         <v>122</v>
       </c>
-      <c r="D22" t="s">
+      <c r="H22" t="s">
         <v>123</v>
-      </c>
-      <c r="E22" t="s">
-        <v>124</v>
-      </c>
-      <c r="F22" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" t="s">
-        <v>125</v>
-      </c>
-      <c r="H22" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" t="s">
+        <v>126</v>
+      </c>
+      <c r="E23" t="s">
+        <v>286</v>
+      </c>
+      <c r="F23" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>122</v>
+      </c>
+      <c r="H23" t="s">
         <v>127</v>
-      </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>128</v>
-      </c>
-      <c r="D23" t="s">
-        <v>129</v>
-      </c>
-      <c r="E23" t="s">
-        <v>130</v>
-      </c>
-      <c r="F23" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" t="s">
-        <v>125</v>
-      </c>
-      <c r="H23" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" t="s">
+        <v>130</v>
+      </c>
+      <c r="E24" t="s">
+        <v>131</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
         <v>132</v>
       </c>
-      <c r="B24" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="H24" t="s">
         <v>133</v>
-      </c>
-      <c r="D24" t="s">
-        <v>134</v>
-      </c>
-      <c r="E24" t="s">
-        <v>135</v>
-      </c>
-      <c r="F24" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" t="s">
-        <v>136</v>
-      </c>
-      <c r="H24" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>135</v>
+      </c>
+      <c r="D25" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" t="s">
+        <v>137</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>132</v>
+      </c>
+      <c r="H25" t="s">
         <v>138</v>
-      </c>
-      <c r="B25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" t="s">
-        <v>139</v>
-      </c>
-      <c r="D25" t="s">
-        <v>140</v>
-      </c>
-      <c r="E25" t="s">
-        <v>141</v>
-      </c>
-      <c r="F25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H25" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>139</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>140</v>
+      </c>
+      <c r="D26" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" t="s">
+        <v>142</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
         <v>143</v>
       </c>
-      <c r="B26" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="H26" t="s">
         <v>144</v>
-      </c>
-      <c r="D26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E26" t="s">
-        <v>146</v>
-      </c>
-      <c r="F26" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" t="s">
-        <v>147</v>
-      </c>
-      <c r="H26" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" t="s">
+        <v>147</v>
+      </c>
+      <c r="E27" t="s">
+        <v>148</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
+        <v>143</v>
+      </c>
+      <c r="H27" t="s">
         <v>149</v>
-      </c>
-      <c r="B27" t="s">
-        <v>22</v>
-      </c>
-      <c r="C27" t="s">
-        <v>150</v>
-      </c>
-      <c r="D27" t="s">
-        <v>151</v>
-      </c>
-      <c r="E27" t="s">
-        <v>152</v>
-      </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" t="s">
-        <v>147</v>
-      </c>
-      <c r="H27" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" t="s">
+        <v>151</v>
+      </c>
+      <c r="D28" t="s">
+        <v>152</v>
+      </c>
+      <c r="E28" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" t="s">
         <v>154</v>
       </c>
-      <c r="B28" t="s">
-        <v>22</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="H28" t="s">
         <v>155</v>
-      </c>
-      <c r="D28" t="s">
-        <v>156</v>
-      </c>
-      <c r="E28" t="s">
-        <v>157</v>
-      </c>
-      <c r="F28" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" t="s">
-        <v>158</v>
-      </c>
-      <c r="H28" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>156</v>
+      </c>
+      <c r="B29" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29" t="s">
+        <v>158</v>
+      </c>
+      <c r="E29" t="s">
+        <v>159</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>154</v>
+      </c>
+      <c r="H29" t="s">
         <v>160</v>
-      </c>
-      <c r="B29" t="s">
-        <v>22</v>
-      </c>
-      <c r="C29" t="s">
-        <v>161</v>
-      </c>
-      <c r="D29" t="s">
-        <v>162</v>
-      </c>
-      <c r="E29" t="s">
-        <v>163</v>
-      </c>
-      <c r="F29" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" t="s">
-        <v>158</v>
-      </c>
-      <c r="H29" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" t="s">
+        <v>163</v>
+      </c>
+      <c r="E30" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" t="s">
         <v>165</v>
       </c>
-      <c r="B30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="H30" t="s">
         <v>166</v>
-      </c>
-      <c r="D30" t="s">
-        <v>167</v>
-      </c>
-      <c r="E30" t="s">
-        <v>168</v>
-      </c>
-      <c r="F30" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" t="s">
-        <v>169</v>
-      </c>
-      <c r="H30" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>167</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" t="s">
+        <v>169</v>
+      </c>
+      <c r="E31" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
+        <v>165</v>
+      </c>
+      <c r="H31" t="s">
         <v>171</v>
-      </c>
-      <c r="B31" t="s">
-        <v>22</v>
-      </c>
-      <c r="C31" t="s">
-        <v>172</v>
-      </c>
-      <c r="D31" t="s">
-        <v>173</v>
-      </c>
-      <c r="E31" t="s">
-        <v>174</v>
-      </c>
-      <c r="F31" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" t="s">
-        <v>169</v>
-      </c>
-      <c r="H31" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>173</v>
+      </c>
+      <c r="D32" t="s">
+        <v>174</v>
+      </c>
+      <c r="E32" t="s">
+        <v>175</v>
+      </c>
+      <c r="F32" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" t="s">
         <v>176</v>
       </c>
-      <c r="B32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="H32" t="s">
         <v>177</v>
-      </c>
-      <c r="D32" t="s">
-        <v>178</v>
-      </c>
-      <c r="E32" t="s">
-        <v>179</v>
-      </c>
-      <c r="F32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" t="s">
-        <v>180</v>
-      </c>
-      <c r="H32" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>178</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>179</v>
+      </c>
+      <c r="D33" t="s">
+        <v>180</v>
+      </c>
+      <c r="E33" t="s">
+        <v>181</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>176</v>
+      </c>
+      <c r="H33" t="s">
         <v>182</v>
-      </c>
-      <c r="B33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
-        <v>183</v>
-      </c>
-      <c r="D33" t="s">
-        <v>184</v>
-      </c>
-      <c r="E33" t="s">
-        <v>185</v>
-      </c>
-      <c r="F33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" t="s">
-        <v>180</v>
-      </c>
-      <c r="H33" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>183</v>
+      </c>
+      <c r="B34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" t="s">
+        <v>184</v>
+      </c>
+      <c r="D34" t="s">
+        <v>185</v>
+      </c>
+      <c r="E34" t="s">
+        <v>186</v>
+      </c>
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" t="s">
         <v>187</v>
       </c>
-      <c r="B34" t="s">
-        <v>22</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="H34" t="s">
         <v>188</v>
-      </c>
-      <c r="D34" t="s">
-        <v>189</v>
-      </c>
-      <c r="E34" t="s">
-        <v>190</v>
-      </c>
-      <c r="F34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" t="s">
-        <v>191</v>
-      </c>
-      <c r="H34" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35" t="s">
+        <v>190</v>
+      </c>
+      <c r="D35" t="s">
+        <v>191</v>
+      </c>
+      <c r="E35" t="s">
+        <v>192</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" t="s">
+        <v>187</v>
+      </c>
+      <c r="H35" t="s">
         <v>193</v>
-      </c>
-      <c r="B35" t="s">
-        <v>22</v>
-      </c>
-      <c r="C35" t="s">
-        <v>194</v>
-      </c>
-      <c r="D35" t="s">
-        <v>195</v>
-      </c>
-      <c r="E35" t="s">
-        <v>196</v>
-      </c>
-      <c r="F35" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" t="s">
-        <v>191</v>
-      </c>
-      <c r="H35" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>194</v>
+      </c>
+      <c r="B36" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36" t="s">
+        <v>195</v>
+      </c>
+      <c r="D36" t="s">
+        <v>196</v>
+      </c>
+      <c r="E36" t="s">
+        <v>197</v>
+      </c>
+      <c r="F36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" t="s">
         <v>198</v>
       </c>
-      <c r="B36" t="s">
-        <v>22</v>
-      </c>
-      <c r="C36" t="s">
+      <c r="H36" t="s">
         <v>199</v>
-      </c>
-      <c r="D36" t="s">
-        <v>200</v>
-      </c>
-      <c r="E36" t="s">
-        <v>201</v>
-      </c>
-      <c r="F36" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" t="s">
-        <v>202</v>
-      </c>
-      <c r="H36" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>200</v>
+      </c>
+      <c r="B37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37" t="s">
+        <v>201</v>
+      </c>
+      <c r="D37" t="s">
+        <v>202</v>
+      </c>
+      <c r="E37" t="s">
+        <v>203</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" t="s">
+        <v>198</v>
+      </c>
+      <c r="H37" t="s">
         <v>204</v>
-      </c>
-      <c r="B37" t="s">
-        <v>22</v>
-      </c>
-      <c r="C37" t="s">
-        <v>205</v>
-      </c>
-      <c r="D37" t="s">
-        <v>206</v>
-      </c>
-      <c r="E37" t="s">
-        <v>207</v>
-      </c>
-      <c r="F37" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" t="s">
-        <v>202</v>
-      </c>
-      <c r="H37" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>205</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" t="s">
+        <v>206</v>
+      </c>
+      <c r="D38" t="s">
+        <v>207</v>
+      </c>
+      <c r="E38" t="s">
+        <v>208</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" t="s">
         <v>209</v>
       </c>
-      <c r="B38" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="H38" t="s">
         <v>210</v>
-      </c>
-      <c r="D38" t="s">
-        <v>211</v>
-      </c>
-      <c r="E38" t="s">
-        <v>212</v>
-      </c>
-      <c r="F38" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" t="s">
-        <v>213</v>
-      </c>
-      <c r="H38" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>211</v>
+      </c>
+      <c r="B39" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s">
+        <v>212</v>
+      </c>
+      <c r="D39" t="s">
+        <v>213</v>
+      </c>
+      <c r="E39" t="s">
+        <v>214</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" t="s">
+        <v>209</v>
+      </c>
+      <c r="H39" t="s">
         <v>215</v>
-      </c>
-      <c r="B39" t="s">
-        <v>22</v>
-      </c>
-      <c r="C39" t="s">
-        <v>216</v>
-      </c>
-      <c r="D39" t="s">
-        <v>217</v>
-      </c>
-      <c r="E39" t="s">
-        <v>218</v>
-      </c>
-      <c r="F39" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" t="s">
-        <v>213</v>
-      </c>
-      <c r="H39" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>216</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" t="s">
+        <v>217</v>
+      </c>
+      <c r="D40" t="s">
+        <v>218</v>
+      </c>
+      <c r="E40" t="s">
+        <v>219</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" t="s">
         <v>220</v>
       </c>
-      <c r="B40" t="s">
-        <v>9</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="H40" t="s">
         <v>221</v>
-      </c>
-      <c r="D40" t="s">
-        <v>222</v>
-      </c>
-      <c r="E40" t="s">
-        <v>223</v>
-      </c>
-      <c r="F40" t="s">
-        <v>13</v>
-      </c>
-      <c r="G40" t="s">
-        <v>224</v>
-      </c>
-      <c r="H40" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>222</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>223</v>
+      </c>
+      <c r="D41" t="s">
+        <v>224</v>
+      </c>
+      <c r="E41" t="s">
+        <v>225</v>
+      </c>
+      <c r="F41" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" t="s">
+        <v>220</v>
+      </c>
+      <c r="H41" t="s">
         <v>226</v>
-      </c>
-      <c r="B41" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" t="s">
-        <v>227</v>
-      </c>
-      <c r="D41" t="s">
-        <v>228</v>
-      </c>
-      <c r="E41" t="s">
-        <v>229</v>
-      </c>
-      <c r="F41" t="s">
-        <v>13</v>
-      </c>
-      <c r="G41" t="s">
-        <v>224</v>
-      </c>
-      <c r="H41" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>227</v>
+      </c>
+      <c r="B42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s">
+        <v>228</v>
+      </c>
+      <c r="D42" t="s">
+        <v>229</v>
+      </c>
+      <c r="E42" t="s">
+        <v>230</v>
+      </c>
+      <c r="F42" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" t="s">
         <v>231</v>
       </c>
-      <c r="B42" t="s">
-        <v>22</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="H42" t="s">
         <v>232</v>
-      </c>
-      <c r="D42" t="s">
-        <v>233</v>
-      </c>
-      <c r="E42" t="s">
-        <v>234</v>
-      </c>
-      <c r="F42" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" t="s">
-        <v>235</v>
-      </c>
-      <c r="H42" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>233</v>
+      </c>
+      <c r="B43" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D43" t="s">
+        <v>235</v>
+      </c>
+      <c r="E43" t="s">
+        <v>236</v>
+      </c>
+      <c r="F43" t="s">
+        <v>12</v>
+      </c>
+      <c r="G43" t="s">
+        <v>231</v>
+      </c>
+      <c r="H43" t="s">
         <v>237</v>
-      </c>
-      <c r="B43" t="s">
-        <v>22</v>
-      </c>
-      <c r="C43" t="s">
-        <v>238</v>
-      </c>
-      <c r="D43" t="s">
-        <v>239</v>
-      </c>
-      <c r="E43" t="s">
-        <v>240</v>
-      </c>
-      <c r="F43" t="s">
-        <v>13</v>
-      </c>
-      <c r="G43" t="s">
-        <v>235</v>
-      </c>
-      <c r="H43" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>238</v>
+      </c>
+      <c r="B44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
+        <v>239</v>
+      </c>
+      <c r="D44" t="s">
+        <v>240</v>
+      </c>
+      <c r="E44" t="s">
+        <v>241</v>
+      </c>
+      <c r="F44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G44" t="s">
         <v>242</v>
       </c>
-      <c r="B44" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="H44" t="s">
         <v>243</v>
-      </c>
-      <c r="D44" t="s">
-        <v>244</v>
-      </c>
-      <c r="E44" t="s">
-        <v>245</v>
-      </c>
-      <c r="F44" t="s">
-        <v>13</v>
-      </c>
-      <c r="G44" t="s">
-        <v>246</v>
-      </c>
-      <c r="H44" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>244</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" t="s">
+        <v>245</v>
+      </c>
+      <c r="D45" t="s">
+        <v>246</v>
+      </c>
+      <c r="E45" t="s">
+        <v>247</v>
+      </c>
+      <c r="F45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G45" t="s">
+        <v>242</v>
+      </c>
+      <c r="H45" t="s">
         <v>248</v>
-      </c>
-      <c r="B45" t="s">
-        <v>22</v>
-      </c>
-      <c r="C45" t="s">
-        <v>249</v>
-      </c>
-      <c r="D45" t="s">
-        <v>250</v>
-      </c>
-      <c r="E45" t="s">
-        <v>251</v>
-      </c>
-      <c r="F45" t="s">
-        <v>13</v>
-      </c>
-      <c r="G45" t="s">
-        <v>246</v>
-      </c>
-      <c r="H45" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>249</v>
+      </c>
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>250</v>
+      </c>
+      <c r="D46" t="s">
+        <v>251</v>
+      </c>
+      <c r="E46" t="s">
+        <v>252</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" t="s">
         <v>253</v>
       </c>
-      <c r="B46" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" t="s">
+      <c r="H46" t="s">
         <v>254</v>
-      </c>
-      <c r="D46" t="s">
-        <v>255</v>
-      </c>
-      <c r="E46" t="s">
-        <v>256</v>
-      </c>
-      <c r="F46" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" t="s">
-        <v>257</v>
-      </c>
-      <c r="H46" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>255</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>256</v>
+      </c>
+      <c r="D47" t="s">
+        <v>257</v>
+      </c>
+      <c r="E47" t="s">
+        <v>258</v>
+      </c>
+      <c r="F47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" t="s">
+        <v>253</v>
+      </c>
+      <c r="H47" t="s">
         <v>259</v>
-      </c>
-      <c r="B47" t="s">
-        <v>9</v>
-      </c>
-      <c r="C47" t="s">
-        <v>260</v>
-      </c>
-      <c r="D47" t="s">
-        <v>261</v>
-      </c>
-      <c r="E47" t="s">
-        <v>262</v>
-      </c>
-      <c r="F47" t="s">
-        <v>13</v>
-      </c>
-      <c r="G47" t="s">
-        <v>257</v>
-      </c>
-      <c r="H47" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>260</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D48" t="s">
+        <v>262</v>
+      </c>
+      <c r="E48" t="s">
+        <v>263</v>
+      </c>
+      <c r="F48" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" t="s">
         <v>264</v>
       </c>
-      <c r="B48" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="H48" t="s">
         <v>265</v>
-      </c>
-      <c r="D48" t="s">
-        <v>266</v>
-      </c>
-      <c r="E48" t="s">
-        <v>267</v>
-      </c>
-      <c r="F48" t="s">
-        <v>13</v>
-      </c>
-      <c r="G48" t="s">
-        <v>268</v>
-      </c>
-      <c r="H48" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>266</v>
+      </c>
+      <c r="B49" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" t="s">
+        <v>267</v>
+      </c>
+      <c r="D49" t="s">
+        <v>268</v>
+      </c>
+      <c r="E49" t="s">
+        <v>269</v>
+      </c>
+      <c r="F49" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" t="s">
+        <v>264</v>
+      </c>
+      <c r="H49" t="s">
         <v>270</v>
-      </c>
-      <c r="B49" t="s">
-        <v>22</v>
-      </c>
-      <c r="C49" t="s">
-        <v>271</v>
-      </c>
-      <c r="D49" t="s">
-        <v>272</v>
-      </c>
-      <c r="E49" t="s">
-        <v>273</v>
-      </c>
-      <c r="F49" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" t="s">
-        <v>268</v>
-      </c>
-      <c r="H49" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>271</v>
+      </c>
+      <c r="B50" t="s">
+        <v>272</v>
+      </c>
+      <c r="C50" t="s">
+        <v>273</v>
+      </c>
+      <c r="D50" t="s">
+        <v>274</v>
+      </c>
+      <c r="E50" t="s">
         <v>275</v>
       </c>
-      <c r="B50" t="s">
+      <c r="F50" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" t="s">
         <v>276</v>
       </c>
-      <c r="C50" t="s">
-        <v>285</v>
-      </c>
-      <c r="D50" t="s">
-        <v>287</v>
-      </c>
-      <c r="E50" t="s">
-        <v>286</v>
-      </c>
-      <c r="F50" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>277</v>
-      </c>
-      <c r="H50" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>278</v>
+      </c>
+      <c r="B51" t="s">
+        <v>272</v>
+      </c>
+      <c r="C51" t="s">
         <v>279</v>
       </c>
-      <c r="B51" t="s">
-        <v>276</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
+        <v>280</v>
+      </c>
+      <c r="E51" t="s">
+        <v>281</v>
+      </c>
+      <c r="F51" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" t="s">
+        <v>282</v>
+      </c>
+      <c r="H51" t="s">
         <v>283</v>
-      </c>
-      <c r="D51" t="s">
-        <v>282</v>
-      </c>
-      <c r="E51" t="s">
-        <v>284</v>
-      </c>
-      <c r="F51" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" t="s">
-        <v>280</v>
-      </c>
-      <c r="H51" t="s">
-        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>